<commit_message>
Actualizaciones de landing page, modal de precios y estilos
</commit_message>
<xml_diff>
--- a/PreciosAsisport.xlsx
+++ b/PreciosAsisport.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\Documents\AsiSportweb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\Documents\EcosistemaSasport\AsiSportweb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{296D6E5B-345B-4223-9586-A6CCF4C960E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB73C072-2C9C-49F7-B2D6-4A95DD295B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="21786" windowHeight="14586" xr2:uid="{00C77B3D-DB7D-4531-AEF1-8C1387FE8C5B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Usuarios</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>Usuarios Adicionales</t>
+  </si>
+  <si>
+    <t>Servicios Adicionales</t>
   </si>
 </sst>
 </file>
@@ -80,7 +83,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$USD]\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$USD]\ #,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -134,7 +137,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -451,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6743AAC6-E50F-42A7-B5D3-BF11521BF748}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="19.46875" customWidth="1"/>
@@ -561,48 +564,56 @@
       </c>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A7" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A8" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B9" s="4">
         <v>5</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C9" s="4">
         <v>5</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D9" s="4">
         <v>7</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E9" s="4">
         <v>7</v>
-      </c>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="4">
-        <v>2</v>
-      </c>
-      <c r="C8" s="4">
-        <v>2</v>
-      </c>
-      <c r="D8" s="4">
-        <v>2</v>
-      </c>
-      <c r="E8" s="4">
-        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4">
+        <v>2</v>
+      </c>
+      <c r="C10" s="4">
+        <v>2</v>
+      </c>
+      <c r="D10" s="4">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A12" t="s">
         <v>8</v>
       </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="G15" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>